<commit_message>
chat 7 Multi-Period Historical Model Construction
</commit_message>
<xml_diff>
--- a/example/DEMO_HK_Trainer.xlsx
+++ b/example/DEMO_HK_Trainer.xlsx
@@ -60,7 +60,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,27 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -124,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,7 +117,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,15 +125,13 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,579 +497,810 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>BAV Excel Trainer</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Complete yellow practice cells in dependency order. Run Check to validate the whole workbook: blank cells stay yellow, correct cells turn green, and incorrect cells turn red. Open the matching Answer Key for the formula/input and Note hint.</t>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Complete each historical schedule left-to-right in dependency order. Each schedule is one modeling concept repeated across fiscal periods. Run Check to validate every yellow cell in the workbook. Open the matching Answer Key for the formula/input and Note hint.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Period scope</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>Cell</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Practice cells</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Effective tax rate (latest fiscal year)</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Revenue historical source link</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>F23</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>B18:F18</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Net interest (latest fiscal year)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Net Income historical source link</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>F24</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>B19:F19</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Effective tax rate</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Condensed Financials</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>B24:F24</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Net interest</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Condensed Financials</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>B25:F25</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Net interest after tax</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>F25</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>B26:F26</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>effective_tax_rate_fy, net_interest_fy</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>NOPAT (latest fiscal year)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>F26</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>net_interest_after_tax_fy</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>B27:F27</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>net_income_link, net_interest_after_tax_fy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Operating working capital assets</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>F29</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>B30:F30</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Operating working capital liabilities</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>F30</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>B31:F31</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Net Operating Working Capital (NOWC)</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>F31</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>B32:F32</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>owca_agg, owcl_agg</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Operating long-term assets</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>F32</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>B33:F33</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Operating long-term liabilities</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>F33</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>B34:F34</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Net operating long-term assets (NOLA)</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>F34</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>B35:F35</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>olta_agg, oltl_agg</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Net Operating Assets (NOA)</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>F35</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>B36:F36</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>nowc_agg, nola_agg</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Financial assets</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>F36</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>B37:F37</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Financial liabilities</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>F37</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>B38:F38</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>F38</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>B39:F39</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>financial_assets_agg, financial_liabilities_agg</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Reformulated equity</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>F39</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>B40:F40</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>noa_agg, net_debt</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Sales Growth</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>ALT DuPont</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>C5:F5</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>revenue_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>NOPAT Margin</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>2021–2025 (5 cells)</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>ALT DuPont</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>B6:F6</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>nopat_fy, revenue_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Return on Net Operating Assets (RNOA)</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>E5</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>C7:F7</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>nopat_fy, noa_agg</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>E6</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>C8:F8</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>net_interest_after_tax_fy, net_debt</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Operating Spread (RNOA − After-tax CoD)</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>E7</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>C9:F9</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>rnoa, after_tax_cod</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Financial leverage (FLEV)</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>E8</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>C10:F10</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>net_debt, equity_reformulated_fy</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>ROE decomposition</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>E9</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>C11:F11</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>rnoa, spread, flev</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Actual ROE</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>2022–2025 (4 cells)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>E10</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>equity_reformulated_fy</t>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>C12:F12</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>net_income_link, equity_reformulated_fy</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1319,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>
@@ -1135,272 +1348,272 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Statement: Income Statement</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="12" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="13" t="n">
         <v>8500</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="13" t="n">
         <v>9200</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="13" t="n">
         <v>10100</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="13" t="n">
         <v>11200</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="13" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Cost of sales</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="14" t="n">
         <v>-3400</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="14" t="n">
         <v>-3680</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>-4040</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>-4480</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="14" t="n">
         <v>-5000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="14" t="n">
         <v>5100</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>5520</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="14" t="n">
         <v>6060</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <v>6720</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <v>7500</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Administrative expenses</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="14" t="n">
         <v>-1700</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>-1840</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>-2020</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="14" t="n">
         <v>-2240</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="14" t="n">
         <v>-2500</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Operating profit</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="14" t="n">
         <v>3400</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>3680</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="14" t="n">
         <v>4040</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="14" t="n">
         <v>4480</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="14" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Finance costs</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="14" t="n">
         <v>-120</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>-130</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>-140</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>-150</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="14" t="n">
         <v>-160</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Finance income</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="14" t="n">
         <v>55</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="14" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Profit before tax</t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="14" t="n">
         <v>3325</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="14" t="n">
         <v>3600</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="14" t="n">
         <v>3955</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="14" t="n">
         <v>4390</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="14" t="n">
         <v>4905</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="14" t="n">
         <v>-565</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="14" t="n">
         <v>-612</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="14" t="n">
         <v>-672</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="14" t="n">
         <v>-746</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="14" t="n">
         <v>-833</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Profit for the year</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="14" t="n">
         <v>2760</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="14" t="n">
         <v>2988</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="14" t="n">
         <v>3283</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="14" t="n">
         <v>3644</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="14" t="n">
         <v>4072</v>
       </c>
     </row>
@@ -1427,338 +1640,338 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Statement: Balance Sheet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="12" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="14" t="n">
         <v>1350</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>1680</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="14" t="n">
         <v>1850</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="14" t="n">
         <v>850</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="14" t="n">
         <v>920</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>1010</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>1120</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="14" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="13" t="n">
         <v>680</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="13" t="n">
         <v>736</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="13" t="n">
         <v>808</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="13" t="n">
         <v>896</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="13" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="14" t="n">
         <v>3200</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>3400</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>3600</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="14" t="n">
         <v>3800</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="14" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="13" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="14" t="n">
         <v>1670</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>1894</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>2282</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>2804</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="14" t="n">
         <v>3500</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="14" t="n">
         <v>8500</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="14" t="n">
         <v>9200</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="14" t="n">
         <v>10100</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="14" t="n">
         <v>11200</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="14" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Trade payables</t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="14" t="n">
         <v>595</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="14" t="n">
         <v>644</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="14" t="n">
         <v>707</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="14" t="n">
         <v>784</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="14" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Bank borrowings</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="14" t="n">
         <v>1400</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="14" t="n">
         <v>1300</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="14" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="14" t="n">
         <v>1305</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="14" t="n">
         <v>1456</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="14" t="n">
         <v>1593</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="14" t="n">
         <v>1716</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="14" t="n">
         <v>1825</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B17" s="15" t="n">
+      <c r="B17" s="14" t="n">
         <v>3400</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="14" t="n">
         <v>3500</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="14" t="n">
         <v>3600</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="14" t="n">
         <v>3700</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="14" t="n">
         <v>3800</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Share capital and reserves</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n">
+      <c r="B18" s="14" t="n">
         <v>5100</v>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="C18" s="14" t="n">
         <v>5700</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="14" t="n">
         <v>6500</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="14" t="n">
         <v>7500</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="14" t="n">
         <v>8700</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Total equity</t>
         </is>
       </c>
-      <c r="B19" s="15" t="n">
+      <c r="B19" s="14" t="n">
         <v>5100</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="14" t="n">
         <v>5700</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="14" t="n">
         <v>6500</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="14" t="n">
         <v>7500</v>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="14" t="n">
         <v>8700</v>
       </c>
     </row>
@@ -1785,184 +1998,184 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Statement: Cash Flow Statement</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="12" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Profit for the year</t>
         </is>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="14" t="n">
         <v>2760</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="14" t="n">
         <v>2988</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="14" t="n">
         <v>3283</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>3644</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="14" t="n">
         <v>4072</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Depreciation and amortisation</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="14" t="n">
         <v>340</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="14" t="n">
         <v>368</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>404</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>448</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="14" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="14" t="n">
         <v>1450</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>1600</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="14" t="n">
         <v>1750</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <v>1930</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <v>2070</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Net cash used in investing activities</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="14" t="n">
         <v>-800</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>-850</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>-900</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="14" t="n">
         <v>-950</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="14" t="n">
         <v>-1000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="14" t="n">
         <v>-500</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>-600</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="14" t="n">
         <v>-700</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="14" t="n">
         <v>-800</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="14" t="n">
         <v>-900</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Net change in cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>180</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="14" t="n">
         <v>170</v>
       </c>
     </row>
@@ -1977,7 +2190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1991,923 +2204,740 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Demo Holdings Limited (DEMO) — Condensed Financials</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BALANCE SHEET CLASSIFICATION</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Classification</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="12" t="n">
         <v>44561</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="12" t="n">
         <v>46022</v>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Financial Asset</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="14" t="n">
         <v>1350</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="14" t="n">
         <v>1680</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <v>1850</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Operating Working Capital Asset</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="14" t="n">
         <v>850</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="14" t="n">
         <v>920</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>1010</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="14" t="n">
         <v>1120</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="14" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Operating Working Capital Asset</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="13" t="n">
         <v>680</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="13" t="n">
         <v>736</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="13" t="n">
         <v>808</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="13" t="n">
         <v>896</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="13" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>3200</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="14" t="n">
         <v>3400</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <v>3600</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <v>3800</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="14" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="13" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>1670</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="14" t="n">
         <v>1894</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="14" t="n">
         <v>2282</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="14" t="n">
         <v>2804</v>
       </c>
-      <c r="G11" s="15" t="n">
+      <c r="G11" s="14" t="n">
         <v>3500</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Trade payables</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Operating Working Capital Liability</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>595</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>644</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>707</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="14" t="n">
         <v>784</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="14" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Bank borrowings</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Financial Liability</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="14" t="n">
         <v>1400</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="14" t="n">
         <v>1300</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="14" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Operating Long-Term Liability</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="14" t="n">
         <v>1305</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="14" t="n">
         <v>1456</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="14" t="n">
         <v>1593</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="14" t="n">
         <v>1716</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="14" t="n">
         <v>1825</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Share capital and reserves</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="14" t="n">
         <v>5100</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="14" t="n">
         <v>5700</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="14" t="n">
         <v>6500</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="14" t="n">
         <v>7500</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G15" s="14" t="n">
         <v>8700</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>CONDENSED INCOME STATEMENT</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="12" t="n">
         <v>44561</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="12" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B18" s="12">
-        <f>'Income Statement'!B16</f>
-        <v/>
-      </c>
-      <c r="C18" s="12">
-        <f>'Income Statement'!C16</f>
-        <v/>
-      </c>
-      <c r="D18" s="12">
-        <f>'Income Statement'!D16</f>
-        <v/>
-      </c>
-      <c r="E18" s="12">
-        <f>'Income Statement'!E16</f>
-        <v/>
-      </c>
-      <c r="F18" s="12">
-        <f>'Income Statement'!F16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Pretax Income</t>
         </is>
       </c>
-      <c r="B19" s="12">
+      <c r="B20" s="11">
         <f>'Income Statement'!B14</f>
         <v/>
       </c>
-      <c r="C19" s="12">
+      <c r="C20" s="11">
         <f>'Income Statement'!C14</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D20" s="11">
         <f>'Income Statement'!D14</f>
         <v/>
       </c>
-      <c r="E19" s="12">
+      <c r="E20" s="11">
         <f>'Income Statement'!E14</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F20" s="11">
         <f>'Income Statement'!F14</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Tax Expense</t>
         </is>
       </c>
-      <c r="B20" s="12">
+      <c r="B21" s="11">
         <f>'Income Statement'!B15</f>
         <v/>
       </c>
-      <c r="C20" s="12">
+      <c r="C21" s="11">
         <f>'Income Statement'!C15</f>
         <v/>
       </c>
-      <c r="D20" s="12">
+      <c r="D21" s="11">
         <f>'Income Statement'!D15</f>
         <v/>
       </c>
-      <c r="E20" s="12">
+      <c r="E21" s="11">
         <f>'Income Statement'!E15</f>
         <v/>
       </c>
-      <c r="F20" s="12">
+      <c r="F21" s="11">
         <f>'Income Statement'!F15</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Interest Expense</t>
         </is>
       </c>
-      <c r="B21" s="12">
+      <c r="B22" s="11">
         <f>'Income Statement'!B12</f>
         <v/>
       </c>
-      <c r="C21" s="12">
+      <c r="C22" s="11">
         <f>'Income Statement'!C12</f>
         <v/>
       </c>
-      <c r="D21" s="12">
+      <c r="D22" s="11">
         <f>'Income Statement'!D12</f>
         <v/>
       </c>
-      <c r="E21" s="12">
+      <c r="E22" s="11">
         <f>'Income Statement'!E12</f>
         <v/>
       </c>
-      <c r="F21" s="12">
+      <c r="F22" s="11">
         <f>'Income Statement'!F12</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Interest Income</t>
         </is>
       </c>
-      <c r="B22" s="12">
+      <c r="B23" s="11">
         <f>'Income Statement'!B13</f>
         <v/>
       </c>
-      <c r="C22" s="12">
+      <c r="C23" s="11">
         <f>'Income Statement'!C13</f>
         <v/>
       </c>
-      <c r="D22" s="12">
+      <c r="D23" s="11">
         <f>'Income Statement'!D13</f>
         <v/>
       </c>
-      <c r="E22" s="12">
+      <c r="E23" s="11">
         <f>'Income Statement'!E13</f>
         <v/>
       </c>
-      <c r="F22" s="12">
+      <c r="F23" s="11">
         <f>'Income Statement'!F13</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Effective Tax Rate</t>
         </is>
       </c>
-      <c r="B23" s="16">
-        <f>IF(B19=0,0,-B20/B19)</f>
-        <v/>
-      </c>
-      <c r="C23" s="16">
-        <f>IF(C19=0,0,-C20/C19)</f>
-        <v/>
-      </c>
-      <c r="D23" s="16">
-        <f>IF(D19=0,0,-D20/D19)</f>
-        <v/>
-      </c>
-      <c r="E23" s="16">
-        <f>IF(E19=0,0,-E20/E19)</f>
-        <v/>
-      </c>
-      <c r="F23" s="17" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Net Interest</t>
         </is>
       </c>
-      <c r="B24" s="15">
-        <f>-(B21+B22)</f>
-        <v/>
-      </c>
-      <c r="C24" s="15">
-        <f>-(C21+C22)</f>
-        <v/>
-      </c>
-      <c r="D24" s="15">
-        <f>-(D21+D22)</f>
-        <v/>
-      </c>
-      <c r="E24" s="15">
-        <f>-(E21+E22)</f>
-        <v/>
-      </c>
-      <c r="F24" s="18" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Net Interest After Tax</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f>B24*(1-B23)</f>
-        <v/>
-      </c>
-      <c r="C25" s="15">
-        <f>C24*(1-C23)</f>
-        <v/>
-      </c>
-      <c r="D25" s="15">
-        <f>D24*(1-D23)</f>
-        <v/>
-      </c>
-      <c r="E25" s="15">
-        <f>E24*(1-E23)</f>
-        <v/>
-      </c>
-      <c r="F25" s="18" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="B26" s="20">
-        <f>B18+B25</f>
-        <v/>
-      </c>
-      <c r="C26" s="20">
-        <f>C18+C25</f>
-        <v/>
-      </c>
-      <c r="D26" s="20">
-        <f>D18+D25</f>
-        <v/>
-      </c>
-      <c r="E26" s="20">
-        <f>E18+E25</f>
-        <v/>
-      </c>
-      <c r="F26" s="21" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>CONDENSED BALANCE SHEET</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Operating Working Capital Assets</t>
         </is>
       </c>
-      <c r="B29" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Asset",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C29" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Asset",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D29" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Asset",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E29" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Asset",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F29" s="18" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Operating Working Capital Liabilities</t>
         </is>
       </c>
-      <c r="B30" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Liability",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C30" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Liability",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D30" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Liability",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E30" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Working Capital Liability",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F30" s="18" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>NOWC</t>
         </is>
       </c>
-      <c r="B31" s="14">
-        <f>B29-B30</f>
-        <v/>
-      </c>
-      <c r="C31" s="14">
-        <f>C29-C30</f>
-        <v/>
-      </c>
-      <c r="D31" s="14">
-        <f>D29-D30</f>
-        <v/>
-      </c>
-      <c r="E31" s="14">
-        <f>E29-E30</f>
-        <v/>
-      </c>
-      <c r="F31" s="21" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="B32" s="20" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
+      <c r="F32" s="20" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>Operating Long-Term Assets</t>
         </is>
       </c>
-      <c r="B32" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Asset",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C32" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Asset",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D32" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Asset",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E32" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Asset",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F32" s="18" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>Operating Long-Term Liabilities</t>
         </is>
       </c>
-      <c r="B33" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Liability",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C33" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Liability",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D33" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Liability",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E33" s="15">
-        <f>SUMIF($B$6:$B$15,"Operating Long-Term Liability",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F33" s="18" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>NOLA</t>
-        </is>
-      </c>
-      <c r="B34" s="14">
-        <f>B32-B33</f>
-        <v/>
-      </c>
-      <c r="C34" s="14">
-        <f>C32-C33</f>
-        <v/>
-      </c>
-      <c r="D34" s="14">
-        <f>D32-D33</f>
-        <v/>
-      </c>
-      <c r="E34" s="14">
-        <f>E32-E33</f>
-        <v/>
-      </c>
-      <c r="F34" s="21" t="n"/>
+      <c r="B34" s="18" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="18" t="n"/>
+      <c r="F34" s="18" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
+          <t>NOLA</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+      <c r="E35" s="20" t="n"/>
+      <c r="F35" s="20" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
           <t>NOA</t>
         </is>
       </c>
-      <c r="B35" s="14">
-        <f>B31+B34</f>
-        <v/>
-      </c>
-      <c r="C35" s="14">
-        <f>C31+C34</f>
-        <v/>
-      </c>
-      <c r="D35" s="14">
-        <f>D31+D34</f>
-        <v/>
-      </c>
-      <c r="E35" s="14">
-        <f>E31+E34</f>
-        <v/>
-      </c>
-      <c r="F35" s="21" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="B36" s="20" t="n"/>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="20" t="n"/>
+      <c r="E36" s="20" t="n"/>
+      <c r="F36" s="20" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Financial Assets</t>
         </is>
       </c>
-      <c r="B36" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Asset",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C36" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Asset",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D36" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Asset",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E36" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Asset",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F36" s="18" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="B37" s="18" t="n"/>
+      <c r="C37" s="18" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>Financial Liabilities</t>
         </is>
       </c>
-      <c r="B37" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Liability",C$6:C$15)</f>
-        <v/>
-      </c>
-      <c r="C37" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Liability",D$6:D$15)</f>
-        <v/>
-      </c>
-      <c r="D37" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Liability",E$6:E$15)</f>
-        <v/>
-      </c>
-      <c r="E37" s="15">
-        <f>SUMIF($B$6:$B$15,"Financial Liability",F$6:F$15)</f>
-        <v/>
-      </c>
-      <c r="F37" s="18" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="B38" s="18" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="B38" s="15">
-        <f>B37-B36</f>
-        <v/>
-      </c>
-      <c r="C38" s="15">
-        <f>C37-C36</f>
-        <v/>
-      </c>
-      <c r="D38" s="15">
-        <f>D37-D36</f>
-        <v/>
-      </c>
-      <c r="E38" s="15">
-        <f>E37-E36</f>
-        <v/>
-      </c>
-      <c r="F38" s="18" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>Equity (NOA - Net Debt)</t>
         </is>
       </c>
-      <c r="B39" s="15">
-        <f>B35-B38</f>
-        <v/>
-      </c>
-      <c r="C39" s="15">
-        <f>C35-C38</f>
-        <v/>
-      </c>
-      <c r="D39" s="15">
-        <f>D35-D38</f>
-        <v/>
-      </c>
-      <c r="E39" s="15">
-        <f>E35-E38</f>
-        <v/>
-      </c>
-      <c r="F39" s="18" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="18" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Reported Equity</t>
         </is>
       </c>
-      <c r="B40" s="15">
+      <c r="B41" s="14">
         <f>'Balance Sheet'!B19</f>
         <v/>
       </c>
-      <c r="C40" s="15">
+      <c r="C41" s="14">
         <f>'Balance Sheet'!C19</f>
         <v/>
       </c>
-      <c r="D40" s="15">
+      <c r="D41" s="14">
         <f>'Balance Sheet'!D19</f>
         <v/>
       </c>
-      <c r="E40" s="15">
+      <c r="E41" s="14">
         <f>'Balance Sheet'!E19</f>
         <v/>
       </c>
-      <c r="F40" s="15">
+      <c r="F41" s="14">
         <f>'Balance Sheet'!F19</f>
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>Total Capital</t>
         </is>
       </c>
-      <c r="B41" s="15">
-        <f>B38+B39</f>
-        <v/>
-      </c>
-      <c r="C41" s="15">
-        <f>C38+C39</f>
-        <v/>
-      </c>
-      <c r="D41" s="15">
-        <f>D38+D39</f>
-        <v/>
-      </c>
-      <c r="E41" s="15">
-        <f>E38+E39</f>
-        <v/>
-      </c>
-      <c r="F41" s="15">
-        <f>F38+F39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="inlineStr">
+      <c r="B42" s="14">
+        <f>B39+B40</f>
+        <v/>
+      </c>
+      <c r="C42" s="14">
+        <f>C39+C40</f>
+        <v/>
+      </c>
+      <c r="D42" s="14">
+        <f>D39+D40</f>
+        <v/>
+      </c>
+      <c r="E42" s="14">
+        <f>E39+E40</f>
+        <v/>
+      </c>
+      <c r="F42" s="14">
+        <f>F39+F40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="B42" s="9">
-        <f>IF(ABS(B39-B40)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="C42" s="9">
-        <f>IF(ABS(C39-C40)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="D42" s="9">
-        <f>IF(ABS(D39-D40)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="E42" s="9">
-        <f>IF(ABS(E39-E40)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="F42" s="9">
-        <f>IF(ABS(F39-F40)&lt;1,"OK","CHECK")</f>
+      <c r="B43" s="8">
+        <f>IF(ABS(B40-B41)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="C43" s="8">
+        <f>IF(ABS(C40-C41)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="D43" s="8">
+        <f>IF(ABS(D40-D41)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="E43" s="8">
+        <f>IF(ABS(E40-E41)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="F43" s="8">
+        <f>IF(ABS(F40-F41)&lt;1,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2927,92 +2957,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Demo Holdings Limited — DuPont Decomposition</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>ROE = RNOA + FLEV × Spread</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="12" t="n">
+        <v>44561</v>
+      </c>
+      <c r="C4" s="12" t="n">
         <v>44926</v>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="D4" s="12" t="n">
         <v>45291</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="E4" s="12" t="n">
         <v>45657</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="F4" s="12" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Sales Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>NOPAT Margin</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>RNOA</t>
         </is>
       </c>
-      <c r="E5" s="22" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>After-tax CoD</t>
         </is>
       </c>
-      <c r="E6" s="17" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="E7" s="23" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="21" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>FLEV</t>
         </is>
       </c>
-      <c r="E8" s="22" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>ROE (decomposed)</t>
         </is>
       </c>
-      <c r="E9" s="24" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Actual ROE</t>
         </is>
       </c>
-      <c r="E10" s="17" t="n"/>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3029,7 +3143,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>
@@ -3050,7 +3164,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>
@@ -3071,7 +3185,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>

</xml_diff>

<commit_message>
Step 8A guided classification judgment
</commit_message>
<xml_diff>
--- a/example/DEMO_HK_Trainer.xlsx
+++ b/example/DEMO_HK_Trainer.xlsx
@@ -13,10 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Statement" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condensed Financials" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALT DuPont" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Bear" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Base" sheetId="8" state="hidden" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Bull" sheetId="9" state="hidden" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Summary" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounting Judgment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Bear" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Base" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Bull" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Summary" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,12 +75,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,6 +118,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -125,13 +127,13 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -509,796 +511,796 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>BAV Excel Trainer</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Complete each historical schedule left-to-right in dependency order. Each schedule is one modeling concept repeated across fiscal periods. Run Check to validate every yellow cell in the workbook. Open the matching Answer Key for the formula/input and Note hint.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Schedule</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Period scope</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Practice cells</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Revenue historical source link</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>B18:F18</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>B19:F19</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Net Income historical source link</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>B19:F19</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>B20:F20</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Effective tax rate</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>B24:F24</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>B25:F25</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Net interest</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>B25:F25</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>B26:F26</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Net interest after tax</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>B26:F26</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>B27:F27</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>effective_tax_rate_fy, net_interest_fy</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>B27:F27</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>B28:F28</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>net_income_link, net_interest_after_tax_fy</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Operating working capital assets</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>B30:F30</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>B31:F31</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Operating working capital liabilities</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>B31:F31</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>B32:F32</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Net Operating Working Capital (NOWC)</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>B32:F32</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>B33:F33</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>owca_agg, owcl_agg</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Operating long-term assets</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>B33:F33</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>B34:F34</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Operating long-term liabilities</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>B34:F34</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>B35:F35</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Net operating long-term assets (NOLA)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>B35:F35</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>B36:F36</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>olta_agg, oltl_agg</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n">
+      <c r="A17" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Net Operating Assets (NOA)</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>B36:F36</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>B37:F37</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>nowc_agg, nola_agg</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Financial assets</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>B37:F37</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>B38:F38</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Financial liabilities</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>B38:F38</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>B39:F39</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n">
+      <c r="A20" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>B39:F39</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>B40:F40</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>financial_assets_agg, financial_liabilities_agg</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="n">
+      <c r="A21" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Reformulated equity</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Condensed Financials</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>B40:F40</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>B41:F41</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>noa_agg, net_debt</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Sales Growth</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>C5:F5</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>revenue_link</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>NOPAT Margin</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>2021–2025 (5 cells)</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>B6:F6</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>nopat_fy, revenue_link</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="n">
+      <c r="A24" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Return on Net Operating Assets (RNOA)</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>C7:F7</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>nopat_fy, noa_agg</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>C8:F8</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>net_interest_after_tax_fy, net_debt</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Operating Spread (RNOA − After-tax CoD)</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>C9:F9</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>rnoa, after_tax_cod</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Financial leverage (FLEV)</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>C10:F10</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>net_debt, equity_reformulated_fy</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>ROE decomposition</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>C11:F11</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>rnoa, spread, flev</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n">
+      <c r="A29" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Actual ROE</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>2022–2025 (4 cells)</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>ALT DuPont</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>C12:F12</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>net_income_link, equity_reformulated_fy</t>
         </is>
@@ -1319,7 +1321,28 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Deferred from historical-only v1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>
@@ -1348,272 +1371,272 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Statement: Income Statement</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>8500</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>9200</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>10100</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="14" t="n">
         <v>11200</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Cost of sales</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>-3400</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="15" t="n">
         <v>-3680</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>-4040</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>-4480</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="15" t="n">
         <v>-5000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="15" t="n">
         <v>5100</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="15" t="n">
         <v>5520</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>6060</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="15" t="n">
         <v>6720</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>7500</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Administrative expenses</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="15" t="n">
         <v>-1700</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>-1840</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>-2020</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <v>-2240</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="15" t="n">
         <v>-2500</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Operating profit</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="15" t="n">
         <v>3400</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>3680</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>4040</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="15" t="n">
         <v>4480</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="15" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Finance costs</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="15" t="n">
         <v>-120</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>-130</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>-140</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>-150</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="15" t="n">
         <v>-160</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Finance income</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="15" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Profit before tax</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="15" t="n">
         <v>3325</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>3600</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <v>3955</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="15" t="n">
         <v>4390</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="15" t="n">
         <v>4905</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="15" t="n">
         <v>-565</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="15" t="n">
         <v>-612</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <v>-672</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="15" t="n">
         <v>-746</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="15" t="n">
         <v>-833</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Profit for the year</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="15" t="n">
         <v>2760</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <v>2988</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <v>3283</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <v>3644</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="15" t="n">
         <v>4072</v>
       </c>
     </row>
@@ -1628,7 +1651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1640,338 +1663,360 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Statement: Balance Sheet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="15" t="n">
         <v>1350</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <v>1680</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="15" t="n">
         <v>1850</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>850</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="15" t="n">
         <v>920</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>1010</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>1120</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="15" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>680</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>736</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>808</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <v>896</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="15" t="n">
         <v>3200</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>3400</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>3600</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <v>3800</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="15" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="15" t="n">
         <v>1670</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>1894</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>2282</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>2804</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="15" t="n">
         <v>3500</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="15" t="n">
         <v>8500</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>9200</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>10100</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="15" t="n">
         <v>11200</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="15" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Trade payables</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="15" t="n">
         <v>595</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>644</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <v>707</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="15" t="n">
         <v>784</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="15" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Bank borrowings</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="15" t="n">
         <v>1400</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <v>1300</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="15" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Operating lease liabilities</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>320</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>340</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>360</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>1305</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>1456</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>1593</v>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>1716</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>1825</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="B17" s="15" t="n">
+        <v>1005</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>1136</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>1253</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>1356</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B18" s="15" t="n">
         <v>3400</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C18" s="15" t="n">
         <v>3500</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D18" s="15" t="n">
         <v>3600</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E18" s="15" t="n">
         <v>3700</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F18" s="15" t="n">
         <v>3800</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Share capital and reserves</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B19" s="15" t="n">
         <v>5100</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C19" s="15" t="n">
         <v>5700</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D19" s="15" t="n">
         <v>6500</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E19" s="15" t="n">
         <v>7500</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F19" s="15" t="n">
         <v>8700</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Total equity</t>
         </is>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B20" s="15" t="n">
         <v>5100</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C20" s="15" t="n">
         <v>5700</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D20" s="15" t="n">
         <v>6500</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E20" s="15" t="n">
         <v>7500</v>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="F20" s="15" t="n">
         <v>8700</v>
       </c>
     </row>
@@ -1998,184 +2043,184 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Company: Demo Holdings Limited (DEMO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Statement: Cash Flow Statement</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Units: HKD in Millions</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Source: manual ingestion (HK)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Profit for the year</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="15" t="n">
         <v>2760</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="15" t="n">
         <v>2988</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>3283</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <v>3644</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="15" t="n">
         <v>4072</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Depreciation and amortisation</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>340</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="15" t="n">
         <v>368</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>404</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>448</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="15" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="15" t="n">
         <v>1450</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="15" t="n">
         <v>1600</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>1750</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="15" t="n">
         <v>1930</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>2070</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Net cash used in investing activities</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="15" t="n">
         <v>-800</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>-850</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>-900</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <v>-950</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="15" t="n">
         <v>-1000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="15" t="n">
         <v>-500</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>-600</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>-700</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="15" t="n">
         <v>-800</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="15" t="n">
         <v>-900</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Net change in cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="15" t="n">
         <v>150</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>150</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>180</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="15" t="n">
         <v>170</v>
       </c>
     </row>
@@ -2190,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2204,359 +2249,379 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Demo Holdings Limited (DEMO) — Condensed Financials</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>BALANCE SHEET CLASSIFICATION</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Classification</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <v>46022</v>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Financial Asset</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>1350</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="15" t="n">
         <v>1680</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="15" t="n">
         <v>1850</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Operating Working Capital Asset</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="15" t="n">
         <v>850</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>920</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <v>1010</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="15" t="n">
         <v>1120</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="15" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Operating Working Capital Asset</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>680</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>736</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="14" t="n">
         <v>808</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <v>896</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="14" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="15" t="n">
         <v>3200</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>3400</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="15" t="n">
         <v>3600</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>3800</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="15" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="G10" s="14" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Operating Long-Term Asset</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>1670</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>1894</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="15" t="n">
         <v>2282</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="15" t="n">
         <v>2804</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="15" t="n">
         <v>3500</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Trade payables</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Operating Working Capital Liability</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>595</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>644</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>707</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="15" t="n">
         <v>784</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="G12" s="15" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Bank borrowings</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Financial Liability</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>1400</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="15" t="n">
         <v>1300</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G13" s="15" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Operating lease liabilities</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Operating Long-Term Liability</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>320</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>340</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>360</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>380</v>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Review: Lease liability concept — operating vs financial judgment</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Operating Long-Term Liability</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n">
-        <v>1305</v>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>1456</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>1593</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>1716</v>
-      </c>
-      <c r="G14" s="14" t="n">
-        <v>1825</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="C15" s="15" t="n">
+        <v>1005</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>1136</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>1253</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>1356</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Share capital and reserves</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <v>5100</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <v>5700</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <v>6500</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F16" s="15" t="n">
         <v>7500</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G16" s="15" t="n">
         <v>8700</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>CONDENSED INCOME STATEMENT</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C18" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D18" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <v>46022</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Net Income</t>
         </is>
       </c>
       <c r="B19" s="16" t="n"/>
@@ -2566,129 +2631,129 @@
       <c r="F19" s="16" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Pretax Income</t>
         </is>
       </c>
-      <c r="B20" s="11">
+      <c r="B21" s="12">
         <f>'Income Statement'!B14</f>
         <v/>
       </c>
-      <c r="C20" s="11">
+      <c r="C21" s="12">
         <f>'Income Statement'!C14</f>
         <v/>
       </c>
-      <c r="D20" s="11">
+      <c r="D21" s="12">
         <f>'Income Statement'!D14</f>
         <v/>
       </c>
-      <c r="E20" s="11">
+      <c r="E21" s="12">
         <f>'Income Statement'!E14</f>
         <v/>
       </c>
-      <c r="F20" s="11">
+      <c r="F21" s="12">
         <f>'Income Statement'!F14</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Tax Expense</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B22" s="12">
         <f>'Income Statement'!B15</f>
         <v/>
       </c>
-      <c r="C21" s="11">
+      <c r="C22" s="12">
         <f>'Income Statement'!C15</f>
         <v/>
       </c>
-      <c r="D21" s="11">
+      <c r="D22" s="12">
         <f>'Income Statement'!D15</f>
         <v/>
       </c>
-      <c r="E21" s="11">
+      <c r="E22" s="12">
         <f>'Income Statement'!E15</f>
         <v/>
       </c>
-      <c r="F21" s="11">
+      <c r="F22" s="12">
         <f>'Income Statement'!F15</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Interest Expense</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B23" s="12">
         <f>'Income Statement'!B12</f>
         <v/>
       </c>
-      <c r="C22" s="11">
+      <c r="C23" s="12">
         <f>'Income Statement'!C12</f>
         <v/>
       </c>
-      <c r="D22" s="11">
+      <c r="D23" s="12">
         <f>'Income Statement'!D12</f>
         <v/>
       </c>
-      <c r="E22" s="11">
+      <c r="E23" s="12">
         <f>'Income Statement'!E12</f>
         <v/>
       </c>
-      <c r="F22" s="11">
+      <c r="F23" s="12">
         <f>'Income Statement'!F12</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Interest Income</t>
         </is>
       </c>
-      <c r="B23" s="11">
+      <c r="B24" s="12">
         <f>'Income Statement'!B13</f>
         <v/>
       </c>
-      <c r="C23" s="11">
+      <c r="C24" s="12">
         <f>'Income Statement'!C13</f>
         <v/>
       </c>
-      <c r="D23" s="11">
+      <c r="D24" s="12">
         <f>'Income Statement'!D13</f>
         <v/>
       </c>
-      <c r="E23" s="11">
+      <c r="E24" s="12">
         <f>'Income Statement'!E13</f>
         <v/>
       </c>
-      <c r="F23" s="11">
+      <c r="F24" s="12">
         <f>'Income Statement'!F13</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Effective Tax Rate</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="17" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Net Interest</t>
         </is>
       </c>
       <c r="B25" s="18" t="n"/>
@@ -2698,252 +2763,264 @@
       <c r="F25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Net Interest</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Net Interest After Tax</t>
         </is>
       </c>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="n"/>
-      <c r="F27" s="20" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>CONDENSED BALANCE SHEET</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Operating Working Capital Assets</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Operating Working Capital Liabilities</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>NOWC</t>
         </is>
       </c>
-      <c r="B32" s="20" t="n"/>
-      <c r="C32" s="20" t="n"/>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="20" t="n"/>
-      <c r="F32" s="20" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="21" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Operating Long-Term Assets</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Operating Long-Term Liabilities</t>
         </is>
       </c>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="18" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>NOLA</t>
         </is>
       </c>
-      <c r="B35" s="20" t="n"/>
-      <c r="C35" s="20" t="n"/>
-      <c r="D35" s="20" t="n"/>
-      <c r="E35" s="20" t="n"/>
-      <c r="F35" s="20" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="B36" s="21" t="n"/>
+      <c r="C36" s="21" t="n"/>
+      <c r="D36" s="21" t="n"/>
+      <c r="E36" s="21" t="n"/>
+      <c r="F36" s="21" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>NOA</t>
         </is>
       </c>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="20" t="n"/>
-      <c r="D36" s="20" t="n"/>
-      <c r="E36" s="20" t="n"/>
-      <c r="F36" s="20" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="B37" s="21" t="n"/>
+      <c r="C37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+      <c r="E37" s="21" t="n"/>
+      <c r="F37" s="21" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Financial Assets</t>
         </is>
       </c>
-      <c r="B37" s="18" t="n"/>
-      <c r="C37" s="18" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Financial Liabilities</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="B39" s="18" t="n"/>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Equity (NOA - Net Debt)</t>
         </is>
       </c>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="B41" s="19" t="n"/>
+      <c r="C41" s="19" t="n"/>
+      <c r="D41" s="19" t="n"/>
+      <c r="E41" s="19" t="n"/>
+      <c r="F41" s="19" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Reported Equity</t>
         </is>
       </c>
-      <c r="B41" s="14">
-        <f>'Balance Sheet'!B19</f>
-        <v/>
-      </c>
-      <c r="C41" s="14">
-        <f>'Balance Sheet'!C19</f>
-        <v/>
-      </c>
-      <c r="D41" s="14">
-        <f>'Balance Sheet'!D19</f>
-        <v/>
-      </c>
-      <c r="E41" s="14">
-        <f>'Balance Sheet'!E19</f>
-        <v/>
-      </c>
-      <c r="F41" s="14">
-        <f>'Balance Sheet'!F19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="B42" s="15">
+        <f>'Balance Sheet'!B20</f>
+        <v/>
+      </c>
+      <c r="C42" s="15">
+        <f>'Balance Sheet'!C20</f>
+        <v/>
+      </c>
+      <c r="D42" s="15">
+        <f>'Balance Sheet'!D20</f>
+        <v/>
+      </c>
+      <c r="E42" s="15">
+        <f>'Balance Sheet'!E20</f>
+        <v/>
+      </c>
+      <c r="F42" s="15">
+        <f>'Balance Sheet'!F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Total Capital</t>
         </is>
       </c>
-      <c r="B42" s="14">
-        <f>B39+B40</f>
-        <v/>
-      </c>
-      <c r="C42" s="14">
-        <f>C39+C40</f>
-        <v/>
-      </c>
-      <c r="D42" s="14">
-        <f>D39+D40</f>
-        <v/>
-      </c>
-      <c r="E42" s="14">
-        <f>E39+E40</f>
-        <v/>
-      </c>
-      <c r="F42" s="14">
-        <f>F39+F40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="B43" s="15">
+        <f>B40+B41</f>
+        <v/>
+      </c>
+      <c r="C43" s="15">
+        <f>C40+C41</f>
+        <v/>
+      </c>
+      <c r="D43" s="15">
+        <f>D40+D41</f>
+        <v/>
+      </c>
+      <c r="E43" s="15">
+        <f>E40+E41</f>
+        <v/>
+      </c>
+      <c r="F43" s="15">
+        <f>F40+F41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="B43" s="8">
-        <f>IF(ABS(B40-B41)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="C43" s="8">
-        <f>IF(ABS(C40-C41)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="D43" s="8">
-        <f>IF(ABS(D40-D41)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="E43" s="8">
-        <f>IF(ABS(E40-E41)&lt;1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="F43" s="8">
-        <f>IF(ABS(F40-F41)&lt;1,"OK","CHECK")</f>
+      <c r="B44" s="9">
+        <f>IF(ABS(B41-B42)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="C44" s="9">
+        <f>IF(ABS(C41-C42)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="D44" s="9">
+        <f>IF(ABS(D41-D42)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="E44" s="9">
+        <f>IF(ABS(E41-E42)&lt;1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>IF(ABS(F41-F42)&lt;1,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Operating Working Capital Asset,Operating Working Capital Liability,Operating Long-Term Asset,Operating Long-Term Liability,Financial Asset,Financial Liability,Equity,Exclude"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2969,164 +3046,164 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Demo Holdings Limited — DuPont Decomposition</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>ROE = RNOA + FLEV × Spread</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="13" t="n">
         <v>44561</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="13" t="n">
         <v>44926</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="13" t="n">
         <v>45291</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="13" t="n">
         <v>45657</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Sales Growth</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>NOPAT Margin</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>RNOA</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="21" t="n"/>
-      <c r="F7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>After-tax CoD</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
-      <c r="F9" s="21" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>FLEV</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>ROE (decomposed)</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="17" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Actual ROE</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3139,17 +3216,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Deferred from historical-only v1</t>
-        </is>
-      </c>
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Accounting Judgment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>The supplied treatment is the model's reference treatment, not a universal accounting truth. Compare it with the listed alternative(s), choose the treatment you would defend, and explain the economic consequence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Supplied model treatment</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Alternative(s) to evaluate</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Your treatment</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Your rationale</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Your consequence explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Operating lease liabilities</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Lease liability operating vs financing</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Operating Long-Term Liability</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Financial Liability</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Operating Long-Term Liability,Financial Liability"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3164,7 +3333,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>
@@ -3185,7 +3354,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Deferred from historical-only v1</t>
         </is>

</xml_diff>